<commit_message>
Leads: 2026-09-27 05:21 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,122 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Roof Replacement in Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>orianroofing.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.orianroofing.com/roof-replacement-los-angeles/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>office@oriancr.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(310) 806-5959</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>roof replacement Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Drain Cleaning Solutions | St. Paul, MN | Ultimate Drain Services</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ultimatedrainservices.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.ultimatedrainservices.com/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>info@ultimatedrainservices.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(651) 451-6001</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>St Paul MN</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>drain cleaning service St Paul MN</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 05:32 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -644,7 +644,6 @@
           <t>https://www.ultimatedrainservices.com/</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>info@ultimatedrainservices.com</t>
@@ -674,6 +673,66 @@
         </is>
       </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Suburban Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>suburbanroofingtx.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://suburbanroofingtx.com/new-braunfels-tx</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Suburban Roofing</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>brooks@suburbanroofingtx.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>830-928-9438</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roofing contractor New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 05:43 UTC (cycle 24)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -738,6 +738,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>JKR Roofing Newark, Delaware</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>jkrroofingrenovations.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://jkrroofingrenovations.com/roofing/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>jkr.roofing2@gmail.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(302) 407-9596</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Newark DE</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>residential roofing company Newark DE</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 05:46 UTC (cycle 26)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -798,6 +798,62 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ally HVAC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>allyac.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://allyac.com/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>hvac@allyac.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>813-544-0082</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Tampa FL</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>HVAC contractor Tampa FL</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 05:53 UTC (cycle 31)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -819,7 +819,6 @@
           <t>https://allyac.com/</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>hvac@allyac.com</t>
@@ -849,6 +848,66 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Angels Cooling LLC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>angelscooling.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://angelscooling.com/heat-pump/heat-pump-installation-replacement-mcallen-tx</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Angel Rodriguez</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>services@angelscooling.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(956) 200-9195</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>McAllen TX</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>heat pump installation McAllen TX</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 06:00 UTC (cycle 36)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -913,6 +913,66 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Pacific Coast Roofing Service | Bay Area Roofers</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pcroofingservice.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://pcroofingservice.com/roofing-contractor-oakland-ca/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Year One</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>pacificcoastroof@aol.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(510) 912-5454</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Oakland CA</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roofing contractor Oakland CA</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 06:01 UTC (cycle 37)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -973,6 +973,62 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Get-R-Done Roofing, Gutters &amp; Siding — Flint, MI</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>getrdoneroofing.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://getrdoneroofing.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>office@getrdoneroofing.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>810-441-1730</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Flint MI</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roof replacement Flint MI</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 06:06 UTC (cycle 40)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -994,7 +994,6 @@
           <t>https://getrdoneroofing.com/</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>office@getrdoneroofing.com</t>
@@ -1024,6 +1023,62 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Local Plumbing Services | MAINLINE PLUMBING</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>mainlineplumbing.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.mainlineplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>mainline@mainlineplumbing.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(206) 294-9691</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Federal Way WA</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>plumbing company Federal Way WA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 06:07 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1049,7 +1049,6 @@
           <t>https://www.mainlineplumbing.com/</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>mainline@mainlineplumbing.com</t>
@@ -1079,6 +1078,62 @@
         </is>
       </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Archer Air Conditioning Service Co., Inc. - Archer Air Conditioning Service Co.,</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>archerac.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.archerac.com/hvac-service-knoxville-tn/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>First Last</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>service@archerac.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Knoxville TN</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>66</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>air conditioning repair Knoxville TN</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 06:23 UTC (cycle 52)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1114,7 +1114,6 @@
           <t>service@archerac.com</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Knoxville TN</t>
@@ -1134,6 +1133,126 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Little Rock, AR | Metal, Copper &amp; Slate Roofing | Sandrock</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>sandrockroofing.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://sandrockroofing.com/service-areas/little-rock</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Arkansas Roofing</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@sandrockroofing.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(501) 391-6080</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Little Rock AR</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>94</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Little Rock AR</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Metal Works Inc - Home</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>metalworksar.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.metalworksar.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Damon Dennis</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>damon@metalworksar.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>501-868-8000</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Little Rock AR</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>84</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Little Rock AR</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 06:26 UTC (cycle 54)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1258,6 +1258,66 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>American Construction Roofing, Siding and Windows</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>amconstruct.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://amconstruct.com/service-area/roofing-contractor-camden-county-nj/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Involvement Our</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>office@amconstruct.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(844) 677-6776</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Camden NJ</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>98</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>roofing contractor Camden NJ</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 06:28 UTC (cycle 55)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1318,6 +1318,62 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Riverside Roofing</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>riversideroofrepair.homes</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://riversideroofrepair.homes/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>info@riversideroofrepair.homes</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1951528001</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Riverside CA</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>roof repair company Riverside CA</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 06:38 UTC (cycle 62)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1339,7 +1339,6 @@
           <t>https://riversideroofrepair.homes/</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>info@riversideroofrepair.homes</t>
@@ -1369,6 +1368,66 @@
         </is>
       </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Great Lakes Roofing &amp; Siding</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>greatlakesroofingmn.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://greatlakesroofingmn.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Siding Fully</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>greatlakesroofingmn@gmail.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(218) 929-0778</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>82</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>residential roofing company Duluth MN</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 06:39 UTC (cycle 63)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1433,6 +1433,62 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Thomas Roofing</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>metalroofbiloxi.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.metalroofbiloxi.com/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofbiloxi.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(888) 990-9411</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Biloxi MS</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>96</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Biloxi MS</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 06:42 UTC (cycle 65)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1454,7 +1454,6 @@
           <t>https://www.metalroofbiloxi.com/</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>moreinfo@metalroofbiloxi.com</t>
@@ -1484,6 +1483,182 @@
         </is>
       </c>
       <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Icy Global Air</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>icyglobalair.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.icyglobalair.com/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>icyglobalairofficial@gmail.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>786-348-3521</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>HVAC contractor Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>R&amp;S Heating and Sheet Metal Inc.</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>rsheatingguys.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://rsheatingguys.com/service-area/salinas-ca/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Rich Russo</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>office@rshvacpros.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(831) 641-0508</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Salinas CA</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>90</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>heating and cooling company Salinas CA</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Reliable AC Services LLC</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>reliableacservices.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://reliableacservices.com/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>South Florida</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>info@reliableacservices.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(561) 929-1133</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>88</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>HVAC contractor Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 06:51 UTC (cycle 71)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1509,7 +1509,6 @@
           <t>https://www.icyglobalair.com/</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>icyglobalairofficial@gmail.com</t>
@@ -1659,6 +1658,62 @@
         </is>
       </c>
       <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PLUMBING SYSTEMS, INC. 859.294.8080</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>plumbingsystemslex.net</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://plumbingsystemslex.net/index.html</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>office@plumbingsystemslex.net</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>859.294.8080</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Lexington KY</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>76</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>plumbing company Lexington KY</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 06:56 UTC (cycle 75)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1684,7 +1684,6 @@
           <t>https://plumbingsystemslex.net/index.html</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>office@plumbingsystemslex.net</t>
@@ -1714,6 +1713,66 @@
         </is>
       </c>
       <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Seaside Plumbing | Wilmington, NC</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>myseasideplumbing.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.myseasideplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Seaside Plumbing</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>myseasideplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(910) 616-6428</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Wilmington NC</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>90</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>plumbing company Wilmington NC</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 07:02 UTC (cycle 79)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1778,6 +1778,66 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Fowler Heating &amp; Air Conditioning, L.L.C. - Madison, WI</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>fowlerheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://fowlerheatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Dane County</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>office.fowlerheating@gmail.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(608) 630-8802</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Madison WI</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>98</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>heating and cooling company Madison WI</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 07:10 UTC (cycle 84)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1838,6 +1838,66 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Today's Plumbing</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>todaysplumbing.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://todaysplumbing.com/service-areas/plumber-in-woodbury-mn/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Twin Cities</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>admin@todaysplumbing.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(763) 308-4706</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Woodbury MN</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>plumber Woodbury MN</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 07:23 UTC (cycle 93)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1898,6 +1898,66 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SN Mechanical</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>snmechanicalhvac.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.snmechanicalhvac.com/furnace-repair-westminster/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Quality Replacement</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>info@snmechanicalhvac.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>(720) 375-6742</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>90</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>furnace repair Westminster CO</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 07:30 UTC (cycle 98)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1958,6 +1958,62 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>My WordPress - Professional Mechanicl HVAC</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>sg-hvacservices.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://sg-hvacservices.com/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>sghvac.office@gmail.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>(917) 825-1556</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Yonkers NY</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>96</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>HVAC contractor Yonkers NY</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 07:40 UTC (cycle 105)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1979,7 +1979,6 @@
           <t>https://sg-hvacservices.com/</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>sghvac.office@gmail.com</t>
@@ -2009,6 +2008,66 @@
         </is>
       </c>
       <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Tioga Plumbing</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>tiogacontractors.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://tiogacontractors.com/sewer-line/sewer-line-emergency-diagnostic-priority-services-frisco-tx</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Popular Schedule</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>dispatch@tiogacontractors.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>817-484-5356</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>90</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>sewer repair Frisco TX</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 07:43 UTC (cycle 107)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2073,6 +2073,66 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Mrgoodguyhvac</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>mrgoodguyhvac.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://mrgoodguyhvac.com/hvac-orem/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Years Of</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>mrgoodguyhvac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>(385) 208-7777</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Orem UT</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>100</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>HVAC contractor Orem UT</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 07:44 UTC (cycle 108)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2133,6 +2133,178 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>South Central Kentucky Heating and Cooling, LLC</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>southcentralkyheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://southcentralkyheatingandcooling.com/bowling-green-ky/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Installation Services</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>scky.hvac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(270) 571-8446</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Bowling Green KY</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>90</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>heating and cooling company Bowling Green KY</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Simonsen Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>simonsenheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://simonsenheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Marty Simonsen</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>contact@sansoxygen.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>(814) 397-1029</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Erie PA</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>76</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>heating and cooling company Erie PA</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>HVAC Doctors</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>hvacdoctorsbg.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://hvacdoctorsbg.com/</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>hvacdoctorsbg@gmail.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Bowling Green KY</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>76</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>heating and cooling company Bowling Green KY</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 07:59 UTC (cycle 118)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2274,13 +2274,11 @@
           <t>https://hvacdoctorsbg.com/</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>hvacdoctorsbg@gmail.com</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>Bowling Green KY</t>
@@ -2300,6 +2298,62 @@
         </is>
       </c>
       <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Carolina Conditions Home Services</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>carolinaconditions.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.carolinaconditions.com/services/hvac/heating/repair/</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>webchat@carolinaconditions.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>803-233-7172</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Columbia SC</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>90</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>furnace repair Columbia SC</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 08:00 UTC (cycle 119)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2324,7 +2324,6 @@
           <t>https://www.carolinaconditions.com/services/hvac/heating/repair/</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>webchat@carolinaconditions.com</t>
@@ -2354,6 +2353,66 @@
         </is>
       </c>
       <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Naples Comfort Systems by Stahlman Cooling &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>stahlmanac.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://stahlmanac.com/air-conditioning/</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Southwest Florid</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>info@stahlmanac.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>239-230-2975</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Naples FL</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>90</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>AC installation Naples FL</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 08:09 UTC (cycle 125)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2418,6 +2418,126 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Discount Roof</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>mydiscountroof.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://mydiscountroof.com/roofing/lafayette/</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Years Serving</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>info@mydiscountroof.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>(219)299-2563</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Lafayette IN</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>100</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>roofing contractor Lafayette IN</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Lafayette, IN | Elite Roofing of Terre Haute</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>eliteroofingterrehaute.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://eliteroofingterrehaute.com/service-areas/lafayette/</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Troy Owner</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>info@eliteroofingterrehaute.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>(812) 234-7285</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Lafayette IN</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>90</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>roofing contractor Lafayette IN</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 08:13 UTC (cycle 128)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2538,6 +2538,66 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>roofmeister.com</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>roofmeister.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://roofmeister.com/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Owner Contact</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>sales@roofmeister.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>(843) 955-0554</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Charleston SC</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>100</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>roofer Charleston SC</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 08:21 UTC (cycle 133)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2598,6 +2598,66 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Marzo Roofing, Inc.</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>marzoroofing.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.marzoroofing.com/roofing-contractor-port-st-lucie/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Port St</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>office@marzoroofing.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>772-871-2489</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>100</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>roofing contractor Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 08:55 UTC (cycle 157)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2658,6 +2658,182 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Balanced Comfort</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>callbalancedcomfort.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://callbalancedcomfort.com/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>info@callbalancedcomfort.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>559-234-4131</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Fresno CA</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>90</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>water heater repair Fresno CA</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Air Care Elite Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>aircareelitehvac.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://aircareelitehvac.com/hvac-services-in-kissimmee-fl/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Cooling From</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>info@aircareelitehvac.com</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>407-443-9004</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>90</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>heating and cooling company Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>thermo Dynamics Solutions</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>thermodynamics-solutions.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://thermodynamics-solutions.com/area-we-serve/kissimmee-fl/</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>rizwan@dijitalroi.com</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>(407) 604-4399</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>90</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>heating and cooling company Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 09:01 UTC (cycle 161)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2679,7 +2679,6 @@
           <t>https://callbalancedcomfort.com/water-heater-repair/</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>info@callbalancedcomfort.com</t>
@@ -2829,6 +2828,66 @@
         </is>
       </c>
       <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>MCM Air</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>mcmair.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://mcmair.com/</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Brochure Schedule</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>service@mcmair.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>920-582-4402</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Oshkosh WI</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>80</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>furnace repair Oshkosh WI</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 09:03 UTC (cycle 162)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2893,6 +2893,66 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Advanced Roofing &amp; Exteriors</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>advancedroofsomaha.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://advancedroofsomaha.com/services/roof-repair/</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Attic Ventila</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>advancedroofingomaha@gmail.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>(402) 609-8072</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Omaha NE</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>100</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>roof repair company Omaha NE</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 09:06 UTC (cycle 164)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2953,6 +2953,62 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Plumber in Riverside, CA 24/7 ⭐⭐⭐⭐⭐ - Fast &amp; Expert</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>riversidecaplumber.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>http://www.riversidecaplumber.com/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>admin@riversidecaplumber.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>(951) 363-2425</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Riverside CA</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>78</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>plumber Riverside CA</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 09:29 UTC (cycle 180)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2974,7 +2974,6 @@
           <t>http://www.riversidecaplumber.com/</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>admin@riversidecaplumber.com</t>
@@ -3004,6 +3003,66 @@
         </is>
       </c>
       <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>FrostBreeze AC Repairs</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>frostbreezeacrepairs.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://frostbreezeacrepairs.com/air-conditioning-repair-in-kissimmee-fl/</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Team The</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>info@frostbreezeacrepairs.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>(407) 439-9910</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>90</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>air conditioning repair Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 09:38 UTC (cycle 186)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3068,6 +3068,66 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Way Cool</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>thewaycoolhvac.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.thewaycoolhvac.com/</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Way Cool</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>milo@thewaycoolhvac.com</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>951-733-2773</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Corona CA</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>86</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>heating and cooling company Corona CA</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 09:39 UTC (cycle 187)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3128,6 +3128,62 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Perfect Climate Heating, Air &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>callperfectclimate.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.callperfectclimate.com/water-heater/water-heater-repair-service-evansville-in</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>info@callperfectclimate.com</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>(812) 615-2733</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Evansville IN</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>90</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>water heater repair Evansville IN</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 09:45 UTC (cycle 191)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3149,7 +3149,6 @@
           <t>https://www.callperfectclimate.com/water-heater/water-heater-repair-service-evansville-in</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>info@callperfectclimate.com</t>
@@ -3179,6 +3178,66 @@
         </is>
       </c>
       <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>draincleaningsummerville.com</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>draincleaningsummerville.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://draincleaningsummerville.com/</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Why Summerville</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>info@draincleaningsummerville.com</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>(854)273-0300</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Summerville SC</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>90</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>drain cleaning service Summerville SC</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 09:48 UTC (cycle 193)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3243,6 +3243,66 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>PSR Roofing Company Of Hollywood | Premium Roofing Contractor</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>psrroofingcompanyofhollywood.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://psrroofingcompanyofhollywood.com/</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Reviews What</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>info@psrroofinghollywood.com</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>(754) 291-4149</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Hollywood FL</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>100</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>residential roofing company Hollywood FL</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 10:05 UTC (cycle 205)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3303,6 +3303,66 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>True Plumb LLC</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>trueplumbtn.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.trueplumbtn.com/</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Need It</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>office@trueplumbtn.com</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>(423) 305-8212</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>90</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>plumber Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 10:07 UTC (cycle 206)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3363,6 +3363,62 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SJP Construction INC | Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>sjpconstructioninc.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://sjpconstructioninc.com/services/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>sjpconstruction89@gmail.com</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>978-905-0471</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Lowell MA</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>84</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Lowell MA</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 10:08 UTC (cycle 207)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3384,7 +3384,6 @@
           <t>https://sjpconstructioninc.com/services/metal-roofing</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>sjpconstruction89@gmail.com</t>
@@ -3414,6 +3413,66 @@
         </is>
       </c>
       <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Peoples Construction</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>peoplesconstruction.info</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://www.peoplesconstruction.info/services/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Nik Gio</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>office@peoplesconstruction.info</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>(945) 274-0387</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Plano TX</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>100</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Plano TX</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 13:47 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3478,6 +3478,66 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>A Quality Roof Now</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>aqualityroofnow.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://aqualityroofnow.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>This Winter</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>info@aqualityroofnow.com</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>(509) 439-1783</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Yakima WA</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>98</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Yakima WA</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 13:51 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3538,6 +3538,126 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Chattanooga Roofing | Compare 5 Free Quotes from Vetted Roofers</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>roofquotes.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://roofquotes.com/chattanooga-tn</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Why Chattanooga</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>hello@roofquotes.com</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>(423) 888-3886</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>90</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>roof replacement Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>JB Air</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>jbair.tech</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://www.jbair.tech/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Schedule Service</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>customerservice@jbair.tech</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>(209) 922-1520</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>74</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>HVAC contractor Stockton CA</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 13:54 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3658,6 +3658,62 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Vance Heating and Air</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>vanceheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://vanceheatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>info@vanceheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>208-530-4942</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Pocatello ID</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>90</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>heat pump installation Pocatello ID</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 13:55 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3679,7 +3679,6 @@
           <t>https://vanceheatingandair.com/</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>info@vanceheatingandair.com</t>
@@ -3709,6 +3708,62 @@
         </is>
       </c>
       <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Newman's Heating &amp; A/C</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>newmanshvac.net</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://newmanshvac.net/city/jersey-city-nj/</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>customer@newmanshvac.net</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>862-520-2790</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Jersey City NJ</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>90</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>AC installation Jersey City NJ</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 13:57 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3734,7 +3734,6 @@
           <t>https://newmanshvac.net/city/jersey-city-nj/</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>customer@newmanshvac.net</t>
@@ -3764,6 +3763,66 @@
         </is>
       </c>
       <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Memphis Air Care</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>memphisair.co</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://www.memphisair.co/services/ac-repair/southaven</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Memphis Air</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>office@memphisaircare.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>901-365-2848</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Southaven MS</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>90</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>air conditioning repair Southaven MS</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:00 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3828,6 +3828,66 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Dream Team Roofing</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>dreamteamroofingfl.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://dreamteamroofingfl.com/locations/roofing-in-miramar</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Get Started</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>info@dreamteamroofingfl.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>(111) 111-1111</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Miramar FL</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>100</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>residential roofing company Miramar FL</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:04 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3888,6 +3888,66 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Newton's Heating &amp; Cooling LLC</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>newtonsheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://newtonsheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Audrey Josh</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>newtonsheatingandcooling@gmail.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>360-448-1414</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>100</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>heating and cooling company Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:06 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3948,6 +3948,66 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Wholesale Roofers</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>wholesaleroofersva.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://www.wholesaleroofersva.com/newportnews</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Wholesale Roofers</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>wholesaleroofers@gmail.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>(757) 424-5981</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Newport News VA</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>90</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>roofer Newport News VA</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:07 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4008,6 +4008,62 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ColdWil HVAC</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>coldwilhvac.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://www.coldwilhvac.com/</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>airconditioning@coldwil.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>(956) 997-9352</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>McAllen TX</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>90</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>HVAC contractor McAllen TX</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:15 UTC (cycle 22)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4029,7 +4029,6 @@
           <t>https://www.coldwilhvac.com/</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>airconditioning@coldwil.com</t>
@@ -4059,6 +4058,66 @@
         </is>
       </c>
       <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Indoor Comfort Team</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>indoorcomfortteam.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://www.indoorcomfortteam.com/</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Financing Discounts</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>info@indoorcomfortteam.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>(314) 230-9542</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>St Louis MO</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>100</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>HVAC contractor St Louis MO</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:19 UTC (cycle 25)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4123,6 +4123,62 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>service.alltechairconditioning.com</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>service.alltechairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://service.alltechairconditioning.com/lp/lawton/heat-pumps/</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>service@alltechokc.com</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>(580) 574-6430</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Lawton OK</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>78</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>heat pump installation Lawton OK</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:25 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4144,7 +4144,6 @@
           <t>https://service.alltechairconditioning.com/lp/lawton/heat-pumps/</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>service@alltechokc.com</t>
@@ -4174,6 +4173,66 @@
         </is>
       </c>
       <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Plumber in Asheville, NC, and Nearby Areas</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>asheville-plumber.com</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://asheville-plumber.com/</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Residential Plumbing</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>ewartplumber@gmail.com</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>(828) 772-6076</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Asheville NC</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>100</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>plumber Asheville NC</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:33 UTC (cycle 35)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4238,6 +4238,66 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Sunrise Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>sunriseheatandcool.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://www.sunriseheatandcool.com/areas-we-serve/yonkers-ny/</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Scott Kelly</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>info@sunriseheatandcool.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>(914) 965-9609</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Yonkers NY</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>100</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>heating and cooling company Yonkers NY</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:35 UTC (cycle 36)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4298,6 +4298,122 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>HomeShield OH</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>homeshieldoh.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://homeshieldoh.com/</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>dbauer@homeshieldoh.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>(614) 333-6705</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Columbus OH</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>96</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>roof repair company Columbus OH</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>AC Repair Coral Springs Pros</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>acrepaircoralsprings.pro</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://acrepaircoralsprings.pro/</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Fernando Hernandez</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>info@acrepaircoralsprings.pro</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>(954) 380-3895</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>84</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>air conditioning repair Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:44 UTC (cycle 42)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4319,7 +4319,6 @@
           <t>https://homeshieldoh.com/</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>dbauer@homeshieldoh.com</t>
@@ -4409,6 +4408,118 @@
         </is>
       </c>
       <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair | Drain Cleaning | Idaho Falls, ID</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>evansplumbingidahofalls.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://www.evansplumbingidahofalls.com/sewer-line-repair</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>service@evansplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>(208) 207-5733</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>100</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>sewer repair Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Sewer Line Repairs | Drain Cleaning | Idaho Falls, ID</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>aaasewerserviceidahofalls.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://www.aaasewerserviceidahofalls.com/sewer-line-repairs</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>contact@aaasewerid.com</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>(208) 243-8422</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>94</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>sewer repair Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:45 UTC (cycle 43)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4434,7 +4434,6 @@
           <t>https://www.evansplumbingidahofalls.com/sewer-line-repair</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>service@evansplumbinginc.com</t>
@@ -4490,7 +4489,6 @@
           <t>https://www.aaasewerserviceidahofalls.com/sewer-line-repairs</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>contact@aaasewerid.com</t>
@@ -4520,6 +4518,66 @@
         </is>
       </c>
       <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Hero's Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>herosheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://herosheatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Values Our</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>example@mail.com</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>(541) 821-1615</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Medford OR</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>100</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>HVAC contractor Medford OR</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:48 UTC (cycle 45)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4583,6 +4583,62 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Plumbing Matters Rooter &amp; Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>plumbingmattersandrooterservices.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://plumbingmattersandrooterservices.com/services/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>services@gmail.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>(909) 714-2207</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Riverside CA</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>100</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>drain cleaning service Riverside CA</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:52 UTC (cycle 48)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4604,7 +4604,6 @@
           <t>https://plumbingmattersandrooterservices.com/services/drain-cleaning/</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>services@gmail.com</t>
@@ -4634,6 +4633,186 @@
         </is>
       </c>
       <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Drain Cleaning in Wichita, KS | Wichita Emergency Drain Cleaning</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>wichitaemergencydraincleaning.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://wichitaemergencydraincleaning.com/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Insured Locally</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>info@wichitaemergencydraincleaning.com</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>(316) 445-9833</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Wichita KS</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>100</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>drain cleaning service Wichita KS</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Focus Plumbing Services, LLC -</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>focusplumbingmn.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://focusplumbingmn.com/</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Plumbing Services</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>focusplumbingmn@gmail.com</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>(651) 295-5417</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>St Paul MN</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>100</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>plumbing company St Paul MN</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Albany Build Pros</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>albanybuildpros.com</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://albanybuildpros.com/</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>See Owner</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>albanybuildpros@gmail.com</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>518-444-3776</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Albany NY</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>100</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>roofing contractor Albany NY</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 14:54 UTC (cycle 49)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4818,6 +4818,122 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Austin Refrigeration &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>austinrefrigeration.us</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://www.austinrefrigeration.us/</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>john@smith.com</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>(800) 803-9202</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Austin TX</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>100</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>HVAC contractor Austin TX</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Trusted Plumbing &amp; Heating Services | Kato Plumbing</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>katoplumbingheating.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://katoplumbingheating.com/</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Your Trusted</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>katoplumbingheating@gmail.com</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>(603) 505-9630</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Manchester NH</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>100</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>plumbing company Manchester NH</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 15:00 UTC (cycle 53)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L77"/>
+  <dimension ref="A1:L78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4839,7 +4839,6 @@
           <t>https://www.austinrefrigeration.us/</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>john@smith.com</t>
@@ -4929,6 +4928,66 @@
         </is>
       </c>
       <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Mountain Range Plumbing</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>mountainrangeplumbing.com</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://mountainrangeplumbing.com/thornton/</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Call Now</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>office@mountainrangeplumbing.com</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>720-990-4599</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Thornton CO</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>100</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>plumbing company Thornton CO</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 15:01 UTC (cycle 54)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L78"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4993,6 +4993,186 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Bickel Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>bickelheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://bickelheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Pedro Meza</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>bickelheatingandcooling@gmail.com</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>(574) 800-4559</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>South Bend IN</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>100</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>heating and cooling company South Bend IN</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Leads Mechanical Services</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>leadsmech.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://leadsmech.com/service-areas/washington-dc/furnace-services/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Furnace Replacement</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>leadsmech@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>240-805-4613</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>84</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>furnace repair Washington DC</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Su'Coy Heating, AC &amp; Duct Cleaning</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>sucoy-hvac.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://sucoy-hvac.com/furnace-repair-service-washington-dc</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Prince George</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>info@sucoy-hvac.com</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>(301) 888 0037</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>80</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>furnace repair Washington DC</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 15:10 UTC (cycle 60)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5173,6 +5173,66 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Metal Roofing in Woodbridge Township, NJ</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>ridgelineremodelinggroup.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://ridgelineremodelinggroup.com/locations/woodbridge-nj/roofing-services/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>No Pressure</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>info@ridgelineremodelinggroup.com</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>(201) 548-3624</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>100</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 15:16 UTC (cycle 64)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5233,6 +5233,66 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Hollywood Plumbing Experts</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>hollywoodplumbingexperts.com</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://hollywoodplumbingexperts.com/</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Aventura Plantation</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>service@hollywoodplumbingexperts.com</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>(754) 240-4741</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Hollywood FL</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>100</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>plumber Hollywood FL</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 15:19 UTC (cycle 66)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5293,6 +5293,66 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Drain Cleaning in Chicago, IL | Precision Today</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>precisiontoday.com</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://www.precisiontoday.com/drain-sewer/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Today Precision</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>info@precisiontoday.com</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>(630) 425-8995</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Chicago IL</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>90</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>drain cleaning service Chicago IL</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 15:25 UTC (cycle 70)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5353,6 +5353,66 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Roofing Services in Olathe, KS - Repairs &amp; Replacements Expert</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>accentroofinggroup.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://www.accentroofinggroup.com/location/olatheks</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Storm Damag</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>luther@accentroofinggroup.com</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>913-219-8972</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Olathe KS</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>100</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>roof replacement Olathe KS</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 15:48 UTC (cycle 86)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5413,6 +5413,66 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>DuraShield Roofing Appleton</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>durashieldroofingappleton.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://durashieldroofingappleton.com/commercial/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Questions Metal</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>info@durashieldroofing.com</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>(920) 738-7663</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Appleton WI</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>100</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Appleton WI</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 15:56 UTC (cycle 91)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5473,6 +5473,66 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>ambroseplumbing</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>ambroseplumbingsewer.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://www.ambroseplumbingsewer.com/</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Extremely Satisfied</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>ambroseplumb@gmail.com</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>630.631.9874</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Naperville IL</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>90</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>plumbing company Naperville IL</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 16:00 UTC (cycle 94)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5533,6 +5533,66 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>AUA HVAC</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>auahvacharrisburg.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://auahvacharrisburg.com/ac-installation/</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Certified Serving</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>hvacaua@gmail.com</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>(717) 343-1224</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Harrisburg PA</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>90</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>AC installation Harrisburg PA</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 16:10 UTC (cycle 101)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5593,6 +5593,66 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Roof Replacement Services in Sacramento | Triple R Roofing</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>triplerroofs.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://triplerroofs.com/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Rogelio Ramirez</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>roofing.tripple.r@gmail.com</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>(916) 420-5635</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Sacramento CA</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>90</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>roof replacement Sacramento CA</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 16:35 UTC (cycle 118)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5653,6 +5653,122 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Jonesboro AR Roofing Company | Rumble Roofing</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>rumbleroofing.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://www.rumbleroofing.com/roofing-jonesboro-ar</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Little Rock</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>hello@rumbleroofing.com</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>(501) 291-1010</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Jonesboro AR</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>90</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>residential roofing company Jonesboro AR</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Metal Roofing- ITM Exterior Solutions</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>itmexteriorsolutions.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://www.itmexteriorsolutions.com/metal</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>david@itmexteriorsolutions.com</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>555-555-5555</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Evansville IN</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>90</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Evansville IN</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 16:40 UTC (cycle 121)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5734,7 +5734,6 @@
           <t>https://www.itmexteriorsolutions.com/metal</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>david@itmexteriorsolutions.com</t>
@@ -5764,6 +5763,66 @@
         </is>
       </c>
       <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>HVAC Company New Jersey</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>heat-pump-installation-edison.aeshvacnj.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://heat-pump-installation-edison.aeshvacnj.com/</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Call Us</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>example@mail.com</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>(888) 978-1291</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Edison NJ</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>100</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>heat pump installation Edison NJ</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 16:46 UTC (cycle 125)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5828,6 +5828,66 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Pipeliners USA</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>pipelinersusa.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://pipelinersusa.com/mesa/</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Up To</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>jake@pipelinersusa.com</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>(480) 535-6503</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Mesa AZ</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>94</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>sewer repair Mesa AZ</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 16:47 UTC (cycle 126)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5888,6 +5888,66 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Roof Replacment Specialist Worcester MA</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>worcester-roofing.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://worcester-roofing.com/roof-replacement.html</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>contact@worcester-roofing.com</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>508-557-2124</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Worcester MA</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>86</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>roof replacement Worcester MA</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 17:17 UTC (cycle 146)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5948,6 +5948,66 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Ernie's Plumbing</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>erniesplumbing.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://erniesplumbing.com/service-areas/grand-prairie</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Tarrant County</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>service@erniesplumbing.com</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>(888) 802-0005</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>100</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>plumbing company Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 17:22 UTC (cycle 150)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6008,6 +6008,66 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Integrated Roofing Systems</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>irsroofingco.com</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://www.irsroofingco.com/roofing-contractor/arvada-co</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Insurance Advocacy</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>info@irsroofingco.com</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>(720) 571-9493</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Arvada CO</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>90</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>roofing contractor Arvada CO</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 17:24 UTC (cycle 151)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6068,6 +6068,62 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Expert Pipe Indy Plumbing</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>expertpipeindy.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://www.expertpipeindy.com/drain-cleaning-repair</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>info@expertpipeindy.com</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>(317) 731-3028</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Carmel IN</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>90</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>drain cleaning service Carmel IN</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 17:25 UTC (cycle 152)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6089,7 +6089,6 @@
           <t>https://www.expertpipeindy.com/drain-cleaning-repair</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>info@expertpipeindy.com</t>
@@ -6119,6 +6118,66 @@
         </is>
       </c>
       <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>AC Install | Chesapeake, VA | Efficient Air</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>yourefficienthvac.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.yourefficienthvac.com/air-conditioning-installation</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Efficient Air</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>bill@yourefficienthvac.com</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2705191873</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Chesapeake VA</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>90</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>AC installation Chesapeake VA</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 17:31 UTC (cycle 156)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6183,6 +6183,66 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Unified Home Remodeling</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>unifiedhomeremodeling.com</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://www.unifiedhomeremodeling.com/roofing-contractor-in-brooklyn-ny/</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Unified Showroom</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>info@unifiedhomeremodeling.com</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>(718) 362-5222</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>100</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>residential roofing company Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 17:34 UTC (cycle 158)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6243,6 +6243,66 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>J Land Contracting</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>jlandgroup.com</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://jlandgroup.com/services/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Land Contracting</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>info@jlandgroup.com</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>(410) 292-0801</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Frederick MD</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>100</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>roof replacement Frederick MD</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 17:51 UTC (cycle 169)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6303,6 +6303,66 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>HVAC Contractor Charleston SC | Alexander</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>alexander-hvac.com</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://www.alexander-hvac.com/</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Cooling Proudly</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>alexanderhvac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>(843) 608-1689</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Charleston SC</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>100</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>HVAC contractor Charleston SC</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 17:54 UTC (cycle 171)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6363,6 +6363,66 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>ThermaFlow Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>thermaflowheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://thermaflowheatingandcooling.com/heat-pump-installation-lakewood-co/</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Team The</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>info@thermaflowheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>(720) 712-7358</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Lakewood CO</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>90</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>heat pump installation Lakewood CO</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 18:05 UTC (cycle 179)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6423,6 +6423,62 @@
         </is>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Metal Roofing in Omaha, NE | H&amp;S Contracting, Inc.</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>hscontractinginc.com</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://www.hscontractinginc.com/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>info@hscontractinginc.com</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>402-554-9994</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Omaha NE</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>90</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Omaha NE</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 18:07 UTC (cycle 180)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6444,7 +6444,6 @@
           <t>https://www.hscontractinginc.com/metal-roofing</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
           <t>info@hscontractinginc.com</t>
@@ -6474,6 +6473,66 @@
         </is>
       </c>
       <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Sutton Brothers Heating, Cooling, Plumbing, &amp; Electrical</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>suttonbros.com</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://suttonbros.com/</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Sutton Brothers</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>info@suttonbros.com</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>336-390-3902</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Greensboro NC</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>90</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>heating and cooling company Greensboro NC</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 18:16 UTC (cycle 186)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6538,6 +6538,66 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Sewer Repairs</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>garlandtx.gov</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://www.garlandtx.gov/3183/Sewer-Repairs</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Helpful Resources</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>garland@garlandtx.gov</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>972-205-3210</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Garland TX</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>98</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>sewer repair Garland TX</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 18:20 UTC (cycle 189)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6598,6 +6598,126 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Roof Replacement | Pittsburgh Roofing Services</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>pittsburghhomerenovation.com</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://www.pittsburghhomerenovation.com/roofing-replacement</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Western Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>sales@thehomerenovationgroup.com</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>412-790-9935</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>90</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>roof replacement Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Tectum Quality Roofing -</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>tectumqualityroofing.com</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://tectumqualityroofing.com/roof-replacement-pittsburgh/</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Get My</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>sales@tectumqualityroofing.com</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>(412) 512-5824</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>90</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>roof replacement Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 18:22 UTC (cycle 190)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6718,6 +6718,66 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Morgantown Plumbers</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>morgantownplumbers.com</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://morgantownplumbers.com/</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Don Knotts</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>info@morgantownplumbers.com</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>(681) 234 5761</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Morgantown WV</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>100</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>plumbing company Morgantown WV</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 21:36 UTC (cycle 45)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6778,6 +6778,118 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Woodbury, MN</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>whitebearheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://www.whitebearheatingandcooling.com/about/service-areas/woodbury/</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>info@whitebearheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>651-426-2044</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Woodbury MN</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>90</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>heating and cooling company Woodbury MN</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Premier Plumbing &amp; Leak Detection</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>premierplumbingandleakdetection.com</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://premierplumbingandleakdetection.com/</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>premierplumbingandleak@gmail.com</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>(352) 219-5880</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Gainesville FL</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>90</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>plumber Gainesville FL</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 21:39 UTC (cycle 47)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:L114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6799,7 +6799,6 @@
           <t>https://www.whitebearheatingandcooling.com/about/service-areas/woodbury/</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
           <t>info@whitebearheatingandcooling.com</t>
@@ -6855,7 +6854,6 @@
           <t>https://premierplumbingandleakdetection.com/</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>premierplumbingandleak@gmail.com</t>
@@ -6885,6 +6883,238 @@
         </is>
       </c>
       <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Keemer Plumbing</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>keemerplumbing.com</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://keemerplumbing.com/west-jordan-ut/</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Keemer Plumbing</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>keemerplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>801-330-5383</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>West Jordan UT</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>100</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>plumber West Jordan UT</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Roof Replacement, Re-Roofing, Installation | Huntsville, AL | Superior Roofing</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>superiorroofinghuntsville.com</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://www.superiorroofinghuntsville.com/</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>info@website.com</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>256-658-8885</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Huntsville AL</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>90</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>roof replacement Huntsville AL</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>F&amp;F Roofing &amp; Construction LLC</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>ffroofingco.com</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://ffroofingco.com/</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>contact@fandfroof.com</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>(812) 470-9993</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Evansville IN</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>88</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>roofing contractor Evansville IN</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Call 4 Handyman Las Vegas</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>call4handymanlasvegas.com</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://call4handymanlasvegas.com/water-heater-repair-henderson-nv/</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>call4handymanlv@gmail.com</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>702-752-0758</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Henderson NV</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>84</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>water heater repair Henderson NV</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 21:40 UTC (cycle 48)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L114"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6969,7 +6969,6 @@
           <t>https://www.superiorroofinghuntsville.com/</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>info@website.com</t>
@@ -7025,7 +7024,6 @@
           <t>https://ffroofingco.com/</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
           <t>contact@fandfroof.com</t>
@@ -7115,6 +7113,62 @@
         </is>
       </c>
       <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Idaho Falls Roofing, Flat Roofing, Metal Roofing, HammerHead Roofing and Constru</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>hammerheadroofingid.com</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://hammerheadroofingid.com/pocatello</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>hammerheadroofsif@gmail.com</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>208-206-5807</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Pocatello ID</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>80</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Pocatello ID</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 21:45 UTC (cycle 51)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7139,7 +7139,6 @@
           <t>https://hammerheadroofingid.com/pocatello</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>hammerheadroofsif@gmail.com</t>
@@ -7169,6 +7168,66 @@
         </is>
       </c>
       <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>The Roof Guru</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>theroofgurus.com</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://theroofgurus.com/amarillo-tx-roofing/</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Why Amarillo</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>info@theroofgurus.com</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>806-203-0974</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Amarillo TX</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>98</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>roof repair company Amarillo TX</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 21:48 UTC (cycle 53)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L116"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7233,6 +7233,62 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Sewer Repair in Aberdeen, SD</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.scottysplumbingandheating.com</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.scottysplumbingandheating.com/sewer-repair/</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>contact@scottysplumbingandheating.com</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>(888) 576-6192</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>90</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>sewer repair Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 21:49 UTC (cycle 54)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L117"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7254,7 +7254,6 @@
           <t>https://aberdeen-sd.scottysplumbingandheating.com/sewer-repair/</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>contact@scottysplumbingandheating.com</t>
@@ -7284,6 +7283,66 @@
         </is>
       </c>
       <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Metal Roofing Bellevue</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>guardianroofingne.com</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://guardianroofingne.com/areas-of-service/bellevue-metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Commercial Roofing</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>abe@guardianroofingne.com</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>(402) 403-9765</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Bellevue NE</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>100</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Bellevue NE</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 21:54 UTC (cycle 57)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7348,6 +7348,302 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>NuShake Roofing</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>nushake.com</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://nushake.com/roofing-companies-stockton-ca/</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Central Valley</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>office@nushake.com</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>(209) 253-0506</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>100</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>residential roofing company Stockton CA</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>EKG Plumbing &amp; Heating | Licensed Brooklyn Plumber &amp; Heating Services – 20+ Year</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>ekgplumbing.com</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://www.ekgplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Team Licensed</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>ekgplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>718-641-4210</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>100</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>plumber Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Stanley Lewis Plumbing and Heating</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>stanleylewisplumbing.com</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://www.stanleylewisplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Alex Lewis</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>services@slph.nyc</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>(718) 774-8757</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>90</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>plumber Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>HVAC Repair, Installation &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>eaglemechanicalllc.com</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://eaglemechanicalllc.com/</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>All Rights</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>tadsit@eaglemechanicalllc.com</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>86</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>HVAC contractor Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Roof Replacement in Fresno, CA | Reasonable Roofing</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>reasonableroofing.net</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://reasonableroofing.net/roof-replacements</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Central Vall</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>reasonableroofing@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>(559) 417-6988</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Fresno CA</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>86</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>roof replacement Fresno CA</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 21:57 UTC (cycle 59)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7559,7 +7559,6 @@
           <t>tadsit@eaglemechanicalllc.com</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr">
         <is>
           <t>Cheyenne WY</t>
@@ -7639,6 +7638,66 @@
         </is>
       </c>
       <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Paloma Plumbing</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>palomaplumbing.com</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://palomaplumbing.com/services/sewer-line-repair</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Fort Worth</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>service@palomatx.com</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>(682) 895-5325</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>90</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>sewer repair Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 22:04 UTC (cycle 64)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L124"/>
+  <dimension ref="A1:L125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7703,6 +7703,66 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>McKinney HVAC</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>mckinneyhvac.com</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://mckinneyhvac.com/collections/heat-pump</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Close Close</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>contact@mckinneyhvac.com</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>469-393-7991</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>McKinney TX</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>90</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>heat pump installation McKinney TX</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 22:20 UTC (cycle 75)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L125"/>
+  <dimension ref="A1:L126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7763,6 +7763,66 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Runway Roofing</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>runwayroofing.com</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://www.runwayroofing.com/carrollton</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Why Carrollton</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>info@runwayroofing.com</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>(469) 819-4183</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Carrollton TX</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>80</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>roofing contractor Carrollton TX</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 22:27 UTC (cycle 80)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L126"/>
+  <dimension ref="A1:L127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7823,6 +7823,66 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>TAC Construction &amp; Roofing</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>tacconstructionandroofing.com</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://tacconstructionandroofing.com/service-areas/pasadena-tx</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>What We</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>tacremodeling@gmail.com</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>(832) 661-6272</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>100</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>roof repair company Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 22:30 UTC (cycle 82)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L127"/>
+  <dimension ref="A1:L128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7883,6 +7883,66 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Emergency Plumber Clarksville</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>sandhillslandsepticservices.com</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://sandhillslandsepticservices.com/emergency-plumber-clarksville-tn/</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Click Here</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>info@sandhillslandsepticservices.com</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>(888) 698-5660</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Clarksville TN</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>90</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>emergency plumber Clarksville TN</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 22:36 UTC (cycle 86)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L128"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7943,6 +7943,66 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Noblehaus Living LLC | Water Heater Repair Overland Park, KS</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>noblehauskc.com</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://noblehauskc.com/Hvac-Contractor/Water-Heater-Repair</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Brian Nelson</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>brian.noblehaus@gmail.com</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>(913) 333-2495</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Overland Park KS</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>82</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>water heater repair Overland Park KS</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 22:42 UTC (cycle 90)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L129"/>
+  <dimension ref="A1:L131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8003,6 +8003,122 @@
         </is>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>911 Water Heater Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>911waterheatersugarland.com</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>https://911waterheatersugarland.com/</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>service@911waterheatersugarland.com</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>281-409-3669</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>100</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>water heater repair Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Water Heater Repair Sugar Land, TX | Same Day Service</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>lonestarwaterheaterpros.com</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>https://lonestarwaterheaterpros.com/sugar-land-tx/water-heater-repair</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Heater Installation</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>info@lonestarwaterheaterpros.com</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>(325) 222-8081</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>84</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>water heater repair Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 22:47 UTC (cycle 94)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L131"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8024,7 +8024,6 @@
           <t>https://911waterheatersugarland.com/</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
           <t>service@911waterheatersugarland.com</t>
@@ -8114,6 +8113,62 @@
         </is>
       </c>
       <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Spire Roofing Solutions - Full Site</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>spireroofingsolutions.com</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>https://www.spireroofingsolutions.com/metal-roofing-1</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>info@spireroofingsolutions.com</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>979-977-3660</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>College Station TX</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>90</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>metal roofing contractor College Station TX</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 22:49 UTC (cycle 95)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L132"/>
+  <dimension ref="A1:L133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8139,7 +8139,6 @@
           <t>https://www.spireroofingsolutions.com/metal-roofing-1</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
           <t>info@spireroofingsolutions.com</t>
@@ -8169,6 +8168,66 @@
         </is>
       </c>
       <c r="L132" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Shield Roofing</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>shieldroofingonline.com</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>https://shieldroofingonline.com/roofing-new-braunfels-tx/</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Roofing Solutions</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>contact@shieldroofingsa.com</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>(210) 348-3680</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>90</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>residential roofing company New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 22:55 UTC (cycle 99)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L133"/>
+  <dimension ref="A1:L134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8233,6 +8233,66 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Roofing Services in Rancho Cucamonga, CA - Superior Roofing</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>superiorroofers.org</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>https://superiorroofers.org/service-areas/rancho-cucamonga-ca</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Rancho Cucamonga</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>hdsuperiorroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>7604881371</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>90</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>roofer Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 23:02 UTC (cycle 104)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L134"/>
+  <dimension ref="A1:L135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8293,6 +8293,66 @@
         </is>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Blue Yeti | HVAC &amp; Plumbing Company | Minneapolis, MN</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>blueyetiservices.com</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://www.blueyetiservices.com/</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Rebates Learn</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>support@blueyetiservices.com</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>952-222-8202</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>100</v>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>plumbing company Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 23:04 UTC (cycle 105)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L135"/>
+  <dimension ref="A1:L136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8353,6 +8353,66 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>HVAC Services in Naples, FL</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>picklerair.com</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://www.picklerair.com/</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Southwest Florid</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>ron@picklerair.com</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>(239) 682-6877</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Naples FL</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>90</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>furnace repair Naples FL</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 23:06 UTC (cycle 107)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L136"/>
+  <dimension ref="A1:L137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8413,6 +8413,66 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Residential Roofing Services | Waco, TX</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>theroofcowaco.com</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>https://www.theroofcowaco.com/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Central Texas</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>info@theroofcowaco.com</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>(254) 236-5764</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Waco TX</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>100</v>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>residential roofing company Waco TX</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 23:21 UTC (cycle 117)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L137"/>
+  <dimension ref="A1:L138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8473,6 +8473,66 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Furnace Everett Pros</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>everettfurnacepros.com</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>https://everettfurnacepros.com/</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Clear Answers</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>everettfurnacepros@gmail.com</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>(425) 380-0422</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Everett WA</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>84</v>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>furnace repair Everett WA</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 23:24 UTC (cycle 119)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L138"/>
+  <dimension ref="A1:L139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8533,6 +8533,62 @@
         </is>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>AmeriRoofs</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>ameriroofs.com</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>https://ameriroofs.com/</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>info@ameriroofs.com</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>410-358-7663</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Baltimore MD</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>76</v>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>roofer Baltimore MD</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 23:33 UTC (cycle 125)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L139"/>
+  <dimension ref="A1:L141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8554,7 +8554,6 @@
           <t>https://ameriroofs.com/</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
           <t>info@ameriroofs.com</t>
@@ -8584,6 +8583,122 @@
         </is>
       </c>
       <c r="L139" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Relentless Roofing Co.</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>relentlessroofingco.com</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>https://relentlessroofingco.com/roof-replacement-south-bend-in/</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Metal Roofing</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>hello@relentlessroofingco.com</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>574-218-0642</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>South Bend IN</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>100</v>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>roof replacement South Bend IN</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Licensed Plumber | Johnson City, TN | David Salts Plumbing</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>davidsaltsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>https://www.davidsaltsplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>plumberman1982@gmail.com</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>423-943-7240</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Johnson City TN</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>90</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>plumber Johnson City TN</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 23:35 UTC (cycle 127)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L141"/>
+  <dimension ref="A1:L142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8669,7 +8669,6 @@
           <t>https://www.davidsaltsplumbing.com/</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
         <is>
           <t>plumberman1982@gmail.com</t>
@@ -8699,6 +8698,66 @@
         </is>
       </c>
       <c r="L141" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Hometown Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>hometownmetalroofing.com</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>https://www.hometownmetalroofing.com/service-areas/rhode-island/cranston</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>New England</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>quotes@hometownmetalroofing.com</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>413-507-0959</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Cranston RI</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>84</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Cranston RI</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 23:50 UTC (cycle 137)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L142"/>
+  <dimension ref="A1:L144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8763,6 +8763,122 @@
         </is>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Wise Builders</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>wisebuildersrnr.com</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>https://wisebuildersrnr.com/biloxi/</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>contact@wisebuildersrnr.com</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>(251) 305-7282</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Biloxi MS</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>100</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>roof replacement Biloxi MS</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Biloxi Roof Replacement | Armor Roofing Gulf Coast</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>armorroofinggulfcoast.com</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>https://www.armorroofinggulfcoast.com/biloxi-roof-replacement</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Scale Exposes</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>info@armorroofinggulfcoast.com</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>(228) 338-3211</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Biloxi MS</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>88</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>roof replacement Biloxi MS</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 23:51 UTC (cycle 138)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L144"/>
+  <dimension ref="A1:L145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8784,7 +8784,6 @@
           <t>https://wisebuildersrnr.com/biloxi/</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
           <t>contact@wisebuildersrnr.com</t>
@@ -8874,6 +8873,66 @@
         </is>
       </c>
       <c r="L144" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Alpine Heating &amp; Air Conditioning -</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>austinalpine.com</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>https://austinalpine.com/</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Experienced Owner</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>info@austinalpine.com</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>(512) 759-4247</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Austin TX</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>100</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>heating and cooling company Austin TX</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-27 23:53 UTC (cycle 139)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L145"/>
+  <dimension ref="A1:L146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8938,6 +8938,66 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Spectrum Roofing &amp; Renovations</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>spectrumroofnola.com</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>https://spectrumroofnola.com/</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Behind Spectrum</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>spectrumroofnola@gmail.com</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>(504) 410-0200</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Metairie LA</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>80</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>roof repair company Metairie LA</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 23:54 UTC (cycle 140)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L146"/>
+  <dimension ref="A1:L148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8998,6 +8998,122 @@
         </is>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Haven Home Remodeling Group</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>havenhrg.com</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>https://www.havenhrg.com/roof-replacement-hollywood</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>South Florida</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>info@havenhrg.com</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>(954) 251-0866</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Hollywood FL</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>100</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>roof replacement Hollywood FL</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Wichita Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>mywichitahvac.com</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>https://mywichitahvac.com/</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>service@mywichitahvac.com</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>316.558.6336</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Wichita KS</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>100</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>heating and cooling company Wichita KS</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-27 23:56 UTC (cycle 141)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-27.xlsx
+++ b/output/leads_2026-09-27.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L148"/>
+  <dimension ref="A1:L149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9079,7 +9079,6 @@
           <t>https://mywichitahvac.com/</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
           <t>service@mywichitahvac.com</t>
@@ -9109,6 +9108,66 @@
         </is>
       </c>
       <c r="L148" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Fleet Plumbing Heating Boiler Repair</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>fleetplumbingandheatingboilerrepair.com</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>https://fleetplumbingandheatingboilerrepair.com/</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Completed Projects</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>info@fleetplumbingandheatingboilerrepair.com</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>(929) 335-9020</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>100</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>water heater repair Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>

</xml_diff>